<commit_message>
Update daily rolling forecast for 2026-09-04
</commit_message>
<xml_diff>
--- a/data/2026_09/snapshots/2026_09_04/dashboard_v3.xlsx
+++ b/data/2026_09/snapshots/2026_09_04/dashboard_v3.xlsx
@@ -491,16 +491,16 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>19003462</v>
+        <v>19026938</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>19752670</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-749208</v>
+        <v>-725732</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-3.8</v>
+        <v>-3.7</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -515,16 +515,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>20961014</v>
+        <v>20984490</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>19752670</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1208344</v>
+        <v>1231820</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -539,13 +539,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>12745092</v>
+        <v>12747788</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>13693510</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-948418</v>
+        <v>-945722</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>-6.9</v>
@@ -563,16 +563,16 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>6050908</v>
+        <v>6071688</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>5869820</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>181088</v>
+        <v>201868</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -611,16 +611,16 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>860</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-2.6</v>
+        <v>-2.4</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -635,16 +635,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>1358</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-24</v>
+        <v>-22</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-1.8</v>
+        <v>-1.6</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>380</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>272</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>13.6</v>
+        <v>14.7</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>高単価型自費 213〜327万円の案件別進捗を確認</t>
+          <t>高単価型自費 215〜330万円の案件別進捗を確認</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>現時点着地見込み 1,900万円は前年同月 1,975万円を下回る見込み（前年差 ▲75万・-3.8%）。一方、通常営業ベース 2,096万円は前年を上回る（+6.1%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
+          <t>現時点着地見込み 1,903万円は前年同月 1,975万円を下回る見込み（前年差 ▲73万・-3.7%）。一方、通常営業ベース 2,098万円は前年を上回る（+6.2%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
         </is>
       </c>
     </row>

</xml_diff>